<commit_message>
Value Model Worksheet: add a currency toggle
Each calc tab now has a currency dropdown (USD/EUR/GBP/CAD/AUD) backed by
a hidden Settings table. A caption, the value-column header, and a
symbol-prefixed display total all update to the selected currency; the
underlying numbers stay currency-neutral so the math is unaffected.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KJa1GsMMHLvb8vFejFkGtX
</commit_message>
<xml_diff>
--- a/public/downloads/procela-governance-value-model.xlsx
+++ b/public/downloads/procela-governance-value-model.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="Start here" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Worked example" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Your value model" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Settings" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet name="Worked example" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Your value model" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,13 +22,25 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0;[Red](#,##0)"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000D1F17"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="006B7A72"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -72,12 +85,6 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="006B7A72"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001F4D38"/>
       <sz val="12"/>
@@ -85,8 +92,8 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="000D1F17"/>
-      <sz val="11"/>
+      <color rgb="002F7052"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="6">
@@ -103,12 +110,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E7F0EB"/>
+        <fgColor rgb="00FFF7E0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF7E0"/>
+        <fgColor rgb="00E7F0EB"/>
       </patternFill>
     </fill>
     <fill>
@@ -126,11 +133,6 @@
       <diagonal/>
     </border>
     <border>
-      <bottom style="thin">
-        <color rgb="00C3CEC8"/>
-      </bottom>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="00D6DEDA"/>
       </left>
@@ -144,59 +146,81 @@
         <color rgb="00D6DEDA"/>
       </bottom>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00C3CEC8"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -562,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B26"/>
+  <dimension ref="B2:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -621,98 +645,102 @@
     <row r="11" ht="30" customHeight="1">
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>3.  Agree the unit economics (Step 1) and operating assumptions (Step 3) with Finance — those three or four numbers are what make the total defensible.</t>
+          <t>3.  Pick your currency from the dropdown at the top of each tab — headers and the total update to match.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>4.  Pull the signals (Step 2) from your catalog: capture them once as a baseline, then re-read them each quarter.</t>
+          <t>4.  Agree the unit economics (Step 1) and operating assumptions (Step 3) with Finance — those few numbers make the total defensible.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>5.  Report the total as a trend, with one line on what moved it. The slope is the story, not the snapshot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="3" t="inlineStr">
+          <t>5.  Pull the signals (Step 2) from your catalog: capture them once as a baseline, then re-read them each quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>6.  Report the total as a trend, with one line on what moved it. The slope is the story, not the snapshot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>The method — three layers</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>•  The un-fakeable signals — classification of sensitive data and owner coverage, computed from the catalog, not asserted on a slide.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>•  The three stories — how each signal maps to risk reduced, cost or time saved, or a decision enabled.</t>
+          <t>•  The un-fakeable signals — classification of sensitive data and owner coverage, computed from the catalog, not asserted on a slide.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="B18" s="4" t="inlineStr">
         <is>
+          <t>•  The three stories — how each signal maps to risk reduced, cost or time saved, or a decision enabled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
           <t>•  The value model — your organisation’s own price on time, incidents, and decisions, agreed with Finance and applied to the signals.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="3" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Rules that keep it credible</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>•  Don’t invent figures. Every euro or dollar comes from an input someone signed off on — change the input, not the credibility.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>•  Baseline before you start. You can only show improvement against a “before”, and today is the cheapest time to capture one.</t>
+          <t>•  Don’t invent figures. Every amount comes from an input someone signed off on — change the input, not the credibility.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>•  Show the slope. Pair the total with its prior value and a one-line “so what”: “at risk fell from X to Y after the billing domain review.”</t>
+          <t>•  Baseline before you start. You can only show improvement against a “before”, and today is the cheapest time to capture one.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="B24" s="4" t="inlineStr">
         <is>
+          <t>•  Show the slope. Pair the total with its prior value and a one-line “so what”: “at risk fell from X to Y after the billing domain review.”</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="B25" s="4" t="inlineStr">
+        <is>
           <t>•  Amber cells are yours to edit. Everything else is a formula that updates when you change an input.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="B26" s="2" t="inlineStr">
+    <row r="27" ht="30" customHeight="1">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>Pair this with the Governance Scorecard Template (procela.ai/resources/scorecard-template) — the same signals belong in front of your governance council.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -723,399 +751,89 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E35"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
-  </cols>
   <sheetData>
-    <row r="2" ht="34" customHeight="1">
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>Worked example</t>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>$</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Illustrative numbers — replace with your own on the “Your value model” tab.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>STEP 1 — Unit economics  (agree these with Finance)</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>£</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>C$</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr"/>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>Loaded cost per analyst hour</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="n">
-        <v>85</v>
-      </c>
-      <c r="E7" s="11" t="inlineStr">
-        <is>
-          <t>Fully-loaded hourly cost of the analysts governance touches</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>Loaded cost per steward / engineer hour</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="n">
-        <v>110</v>
-      </c>
-      <c r="E8" s="11" t="inlineStr">
-        <is>
-          <t>For audit-prep and remediation time</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Expected cost of a reportable data incident</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="n">
-        <v>250000</v>
-      </c>
-      <c r="E9" s="11" t="inlineStr">
-        <is>
-          <t>Fully loaded: fines, response, notification, reputation</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Value of a day saved in a key decision cycle</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E10" s="11" t="inlineStr">
-        <is>
-          <t>What a faster, confident decision is worth per day</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>STEP 2 — Governance signals  (read from your catalog)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>Signal</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>Baseline</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>Current</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>Sensitive data classified</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D14" s="12" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="E14" s="11" t="inlineStr">
-        <is>
-          <t>% of sensitive assets with a classification</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Tier-1 coverage — owned</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="D15" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="11" t="inlineStr">
-        <is>
-          <t>% of tier-1 domains &amp; assets with a named owner</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>STEP 3 — Operating assumptions  (agree these too)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr"/>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>Annual incident probability — baseline exposure</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="E19" s="11" t="inlineStr">
-        <is>
-          <t>Modeled likelihood per year when sensitive data is largely ungoverned</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>Annual incident probability — full coverage (floor)</t>
-        </is>
-      </c>
-      <c r="C20" s="12" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>Irreducible residual even with strong governance</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>Analyst-hours saved per month (at current coverage)</t>
-        </is>
-      </c>
-      <c r="C21" s="13" t="n">
-        <v>40</v>
-      </c>
-      <c r="E21" s="11" t="inlineStr">
-        <is>
-          <t>Less time hunting for owners and re-pulling data</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>Audit-prep hours saved per audit</t>
-        </is>
-      </c>
-      <c r="C22" s="13" t="n">
-        <v>120</v>
-      </c>
-      <c r="E22" s="11" t="inlineStr">
-        <is>
-          <t>Prep becomes a query, not a project</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>Audits per year</t>
-        </is>
-      </c>
-      <c r="C23" s="13" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>Decision-days saved per year</t>
-        </is>
-      </c>
-      <c r="C24" s="13" t="n">
-        <v>20</v>
-      </c>
-      <c r="E24" s="11" t="inlineStr">
-        <is>
-          <t>Faster, confident decisions on trusted, traceable figures</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>THE VALUE  (annual — computed from your inputs)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>Story</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>Annual value</t>
-        </is>
-      </c>
-      <c r="D27" s="8" t="inlineStr"/>
-      <c r="E27" s="8" t="inlineStr">
-        <is>
-          <t>How it’s computed</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>Risk reduced</t>
-        </is>
-      </c>
-      <c r="C28" s="14">
-        <f>C9*(C19-C20)*(D14-C14)</f>
-        <v/>
-      </c>
-      <c r="E28" s="11" t="inlineStr">
-        <is>
-          <t>Incident cost × exposure-driven drop in annual probability</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>Cost &amp; time saved</t>
-        </is>
-      </c>
-      <c r="C29" s="14">
-        <f>C21*12*C7 + C22*C23*C8</f>
-        <v/>
-      </c>
-      <c r="E29" s="11" t="inlineStr">
-        <is>
-          <t>Analyst hours + audit-prep hours, at your loaded rates</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>Decisions enabled</t>
-        </is>
-      </c>
-      <c r="C30" s="14">
-        <f>C24*C10</f>
-        <v/>
-      </c>
-      <c r="E30" s="11" t="inlineStr">
-        <is>
-          <t>Decision-days saved × value per day</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="26" customHeight="1">
-      <c r="B32" s="15" t="inlineStr">
-        <is>
-          <t>TOTAL annual governance value</t>
-        </is>
-      </c>
-      <c r="C32" s="16">
-        <f>SUM(C28:C30)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="17" t="inlineStr">
-        <is>
-          <t>Every figure above traces to an input you set — change an assumption and the total updates. Procela invents no numbers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="17" t="inlineStr">
-        <is>
-          <t>Report it as a trend: “governance value rose from €X to €Y this quarter after the billing and metering domains were reviewed.”</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AUD</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>A$</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>This sheet powers the currency dropdown on each tab. Add rows above to offer more currencies.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="B35:E35"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B34:E34"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1126,7 +844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E35"/>
+  <dimension ref="B2:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1134,363 +852,838 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="52" customWidth="1" min="5" max="5"/>
+    <col hidden="1" width="6" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="2" ht="34" customHeight="1">
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Worked example</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Illustrative numbers — replace with your own on the “Your value model” tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D5" s="10">
+        <f>CONCATENATE("All amounts below are in ",C5," (",G5,") — change it at left")</f>
+        <v/>
+      </c>
+      <c r="G5" s="11">
+        <f>VLOOKUP(C5,Settings!$A$2:$B$6,2,FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>STEP 1 — Unit economics  (agree these with Finance)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr"/>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>Loaded cost per analyst hour</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="n">
+        <v>85</v>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>Fully-loaded hourly cost of the analysts governance touches</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Loaded cost per steward / engineer hour</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="n">
+        <v>110</v>
+      </c>
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>For audit-prep and remediation time</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>Expected cost of a reportable data incident</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="n">
+        <v>250000</v>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>Fully loaded: fines, response, notification, reputation</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>Value of a day saved in a key decision cycle</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>What a faster, confident decision is worth per day</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>STEP 2 — Governance signals  (read from your catalog)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>Sensitive data classified</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D16" s="17" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>% of sensitive assets with a classification</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Tier-1 coverage — owned</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="D17" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>% of tier-1 domains &amp; assets with a named owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>STEP 3 — Operating assumptions  (agree these too)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr"/>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>Annual incident probability — baseline exposure</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E21" s="16" t="inlineStr">
+        <is>
+          <t>Modeled likelihood per year when sensitive data is largely ungoverned</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>Annual incident probability — full coverage (floor)</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E22" s="16" t="inlineStr">
+        <is>
+          <t>Irreducible residual even with strong governance</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Analyst-hours saved per month (at current coverage)</t>
+        </is>
+      </c>
+      <c r="C23" s="18" t="n">
+        <v>40</v>
+      </c>
+      <c r="E23" s="16" t="inlineStr">
+        <is>
+          <t>Less time hunting for owners and re-pulling data</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>Audit-prep hours saved per audit</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="n">
+        <v>120</v>
+      </c>
+      <c r="E24" s="16" t="inlineStr">
+        <is>
+          <t>Prep becomes a query, not a project</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>Audits per year</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>Decision-days saved per year</t>
+        </is>
+      </c>
+      <c r="C26" s="18" t="n">
+        <v>20</v>
+      </c>
+      <c r="E26" s="16" t="inlineStr">
+        <is>
+          <t>Faster, confident decisions on trusted, traceable figures</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>THE VALUE  (annual — computed from your inputs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="19" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C29" s="20">
+        <f>CONCATENATE("Annual value (",C5,")")</f>
+        <v/>
+      </c>
+      <c r="E29" s="19" t="inlineStr">
+        <is>
+          <t>How it’s computed</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Risk reduced</t>
+        </is>
+      </c>
+      <c r="C30" s="21">
+        <f>C11*(C21-C22)*(D16-C16)</f>
+        <v/>
+      </c>
+      <c r="E30" s="16" t="inlineStr">
+        <is>
+          <t>Incident cost × exposure-driven drop in annual probability</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Cost &amp; time saved</t>
+        </is>
+      </c>
+      <c r="C31" s="21">
+        <f>C23*12*C9 + C24*C25*C10</f>
+        <v/>
+      </c>
+      <c r="E31" s="16" t="inlineStr">
+        <is>
+          <t>Analyst hours + audit-prep hours, at your loaded rates</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>Decisions enabled</t>
+        </is>
+      </c>
+      <c r="C32" s="21">
+        <f>C26*C12</f>
+        <v/>
+      </c>
+      <c r="E32" s="16" t="inlineStr">
+        <is>
+          <t>Decision-days saved × value per day</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="26" customHeight="1">
+      <c r="B34" s="22" t="inlineStr">
+        <is>
+          <t>TOTAL annual governance value</t>
+        </is>
+      </c>
+      <c r="C34" s="23">
+        <f>SUM(C30:C32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Shown in selected currency</t>
+        </is>
+      </c>
+      <c r="C35" s="24">
+        <f>CONCATENATE(G5,TEXT(C34,"#,##0"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>Every figure above traces to an input you set — change an assumption (or the currency) and the total updates. Procela invents no numbers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Report it as a trend: “governance value rose from X to Y this quarter after the billing and metering domains were reviewed.”</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B14:E14"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="C5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>Settings!$A$2:$A$6</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:G38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col hidden="1" width="6" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="34" customHeight="1">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Your value model</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Replace the amber cells. Blue results update automatically.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="B5" s="7" t="inlineStr">
+    <row r="5">
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D5" s="10">
+        <f>CONCATENATE("All amounts below are in ",C5," (",G5,") — change it at left")</f>
+        <v/>
+      </c>
+      <c r="G5" s="11">
+        <f>VLOOKUP(C5,Settings!$A$2:$B$6,2,FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>STEP 1 — Unit economics  (agree these with Finance)</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="B6" s="8" t="inlineStr">
+    <row r="8">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr"/>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="D8" s="13" t="inlineStr"/>
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="9" t="inlineStr">
+    <row r="9" ht="22" customHeight="1">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>Loaded cost per analyst hour</t>
         </is>
       </c>
-      <c r="C7" s="10" t="n"/>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="C9" s="15" t="n"/>
+      <c r="E9" s="16" t="inlineStr">
         <is>
           <t>Fully-loaded hourly cost of the analysts governance touches</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="9" t="inlineStr">
+    <row r="10" ht="22" customHeight="1">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>Loaded cost per steward / engineer hour</t>
         </is>
       </c>
-      <c r="C8" s="10" t="n"/>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="C10" s="15" t="n"/>
+      <c r="E10" s="16" t="inlineStr">
         <is>
           <t>For audit-prep and remediation time</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="9" t="inlineStr">
+    <row r="11" ht="22" customHeight="1">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>Expected cost of a reportable data incident</t>
         </is>
       </c>
-      <c r="C9" s="10" t="n"/>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="C11" s="15" t="n"/>
+      <c r="E11" s="16" t="inlineStr">
         <is>
           <t>Fully loaded: fines, response, notification, reputation</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="9" t="inlineStr">
+    <row r="12" ht="22" customHeight="1">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>Value of a day saved in a key decision cycle</t>
         </is>
       </c>
-      <c r="C10" s="10" t="n"/>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="C12" s="15" t="n"/>
+      <c r="E12" s="16" t="inlineStr">
         <is>
           <t>What a faster, confident decision is worth per day</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="B12" s="7" t="inlineStr">
+    <row r="14" ht="24" customHeight="1">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>STEP 2 — Governance signals  (read from your catalog)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="8" t="inlineStr">
+    <row r="15">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C15" s="13" t="inlineStr">
         <is>
           <t>Baseline</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>Current</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E15" s="13" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="9" t="inlineStr">
+    <row r="16" ht="22" customHeight="1">
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>Sensitive data classified</t>
         </is>
       </c>
-      <c r="C14" s="12" t="n"/>
-      <c r="D14" s="12" t="n"/>
-      <c r="E14" s="11" t="inlineStr">
+      <c r="C16" s="17" t="n"/>
+      <c r="D16" s="17" t="n"/>
+      <c r="E16" s="16" t="inlineStr">
         <is>
           <t>% of sensitive assets with a classification</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="B15" s="9" t="inlineStr">
+    <row r="17" ht="22" customHeight="1">
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>Tier-1 coverage — owned</t>
         </is>
       </c>
-      <c r="C15" s="12" t="n"/>
-      <c r="D15" s="12" t="n"/>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="C17" s="17" t="n"/>
+      <c r="D17" s="17" t="n"/>
+      <c r="E17" s="16" t="inlineStr">
         <is>
           <t>% of tier-1 domains &amp; assets with a named owner</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="B17" s="7" t="inlineStr">
+    <row r="19" ht="24" customHeight="1">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>STEP 3 — Operating assumptions  (agree these too)</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="8" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C20" s="13" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr"/>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="D20" s="13" t="inlineStr"/>
+      <c r="E20" s="13" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="B19" s="9" t="inlineStr">
+    <row r="21" ht="22" customHeight="1">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>Annual incident probability — baseline exposure</t>
         </is>
       </c>
-      <c r="C19" s="12" t="n"/>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="C21" s="17" t="n"/>
+      <c r="E21" s="16" t="inlineStr">
         <is>
           <t>Modeled likelihood per year when sensitive data is largely ungoverned</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="9" t="inlineStr">
+    <row r="22" ht="22" customHeight="1">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>Annual incident probability — full coverage (floor)</t>
         </is>
       </c>
-      <c r="C20" s="12" t="n"/>
-      <c r="E20" s="11" t="inlineStr">
+      <c r="C22" s="17" t="n"/>
+      <c r="E22" s="16" t="inlineStr">
         <is>
           <t>Irreducible residual even with strong governance</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="B21" s="9" t="inlineStr">
+    <row r="23" ht="22" customHeight="1">
+      <c r="B23" s="14" t="inlineStr">
         <is>
           <t>Analyst-hours saved per month (at current coverage)</t>
         </is>
       </c>
-      <c r="C21" s="13" t="n"/>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="C23" s="18" t="n"/>
+      <c r="E23" s="16" t="inlineStr">
         <is>
           <t>Less time hunting for owners and re-pulling data</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="B22" s="9" t="inlineStr">
+    <row r="24" ht="22" customHeight="1">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>Audit-prep hours saved per audit</t>
         </is>
       </c>
-      <c r="C22" s="13" t="n"/>
-      <c r="E22" s="11" t="inlineStr">
+      <c r="C24" s="18" t="n"/>
+      <c r="E24" s="16" t="inlineStr">
         <is>
           <t>Prep becomes a query, not a project</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="B23" s="9" t="inlineStr">
+    <row r="25" ht="22" customHeight="1">
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>Audits per year</t>
         </is>
       </c>
-      <c r="C23" s="13" t="n"/>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="B24" s="9" t="inlineStr">
+      <c r="C25" s="18" t="n"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>Decision-days saved per year</t>
         </is>
       </c>
-      <c r="C24" s="13" t="n"/>
-      <c r="E24" s="11" t="inlineStr">
+      <c r="C26" s="18" t="n"/>
+      <c r="E26" s="16" t="inlineStr">
         <is>
           <t>Faster, confident decisions on trusted, traceable figures</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="B26" s="7" t="inlineStr">
+    <row r="28" ht="24" customHeight="1">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>THE VALUE  (annual — computed from your inputs)</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="8" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="19" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>Annual value</t>
-        </is>
-      </c>
-      <c r="D27" s="8" t="inlineStr"/>
-      <c r="E27" s="8" t="inlineStr">
+      <c r="C29" s="20">
+        <f>CONCATENATE("Annual value (",C5,")")</f>
+        <v/>
+      </c>
+      <c r="E29" s="19" t="inlineStr">
         <is>
           <t>How it’s computed</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="B28" s="9" t="inlineStr">
+    <row r="30" ht="22" customHeight="1">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>Risk reduced</t>
         </is>
       </c>
-      <c r="C28" s="14">
-        <f>C9*(C19-C20)*(D14-C14)</f>
+      <c r="C30" s="21">
+        <f>C11*(C21-C22)*(D16-C16)</f>
         <v/>
       </c>
-      <c r="E28" s="11" t="inlineStr">
+      <c r="E30" s="16" t="inlineStr">
         <is>
           <t>Incident cost × exposure-driven drop in annual probability</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="B29" s="9" t="inlineStr">
+    <row r="31" ht="22" customHeight="1">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>Cost &amp; time saved</t>
         </is>
       </c>
-      <c r="C29" s="14">
-        <f>C21*12*C7 + C22*C23*C8</f>
+      <c r="C31" s="21">
+        <f>C23*12*C9 + C24*C25*C10</f>
         <v/>
       </c>
-      <c r="E29" s="11" t="inlineStr">
+      <c r="E31" s="16" t="inlineStr">
         <is>
           <t>Analyst hours + audit-prep hours, at your loaded rates</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="B30" s="9" t="inlineStr">
+    <row r="32" ht="22" customHeight="1">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>Decisions enabled</t>
         </is>
       </c>
-      <c r="C30" s="14">
-        <f>C24*C10</f>
+      <c r="C32" s="21">
+        <f>C26*C12</f>
         <v/>
       </c>
-      <c r="E30" s="11" t="inlineStr">
+      <c r="E32" s="16" t="inlineStr">
         <is>
           <t>Decision-days saved × value per day</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="26" customHeight="1">
-      <c r="B32" s="15" t="inlineStr">
+    <row r="34" ht="26" customHeight="1">
+      <c r="B34" s="22" t="inlineStr">
         <is>
           <t>TOTAL annual governance value</t>
         </is>
       </c>
-      <c r="C32" s="16">
-        <f>SUM(C28:C30)</f>
+      <c r="C34" s="23">
+        <f>SUM(C30:C32)</f>
         <v/>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" s="17" t="inlineStr">
-        <is>
-          <t>Every figure above traces to an input you set — change an assumption and the total updates. Procela invents no numbers.</t>
-        </is>
-      </c>
-    </row>
     <row r="35">
-      <c r="B35" s="17" t="inlineStr">
-        <is>
-          <t>Report it as a trend: “governance value rose from €X to €Y this quarter after the billing and metering domains were reviewed.”</t>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Shown in selected currency</t>
+        </is>
+      </c>
+      <c r="C35" s="24">
+        <f>CONCATENATE(G5,TEXT(C34,"#,##0"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>Every figure above traces to an input you set — change an assumption (or the currency) and the total updates. Procela invents no numbers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Report it as a trend: “governance value rose from X to Y this quarter after the billing and metering domains were reviewed.”</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="B35:E35"/>
-    <mergeCell ref="B12:E12"/>
+  <mergeCells count="9">
+    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="B7:E7"/>
     <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B5:E5"/>
     <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B14:E14"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="C5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>Settings!$A$2:$A$6</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>